<commit_message>
AZT. OL CR:c|high|missing. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/AUSS.OL.xlsx
+++ b/data/obx_xlsx/AUSS.OL.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="471">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Depreciation of right-of-use assets</t>
+  </si>
+  <si>
+    <t>Depreciation (do not use)</t>
   </si>
   <si>
     <t>Impairment</t>
@@ -1621,6 +1624,9 @@
     <xf borderId="3" fillId="0" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="5" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1634,9 +1640,6 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -3164,17 +3167,39 @@
       <c r="K32" s="15">
         <v>709.0</v>
       </c>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="14"/>
-      <c r="O32" s="14"/>
-      <c r="P32" s="14"/>
-      <c r="Q32" s="14"/>
-      <c r="R32" s="14"/>
-      <c r="S32" s="14"/>
-      <c r="T32" s="14"/>
-      <c r="U32" s="14"/>
-      <c r="V32" s="14"/>
+      <c r="L32" s="15">
+        <v>611.0</v>
+      </c>
+      <c r="M32" s="15">
+        <v>566.17</v>
+      </c>
+      <c r="N32" s="15">
+        <v>504.6</v>
+      </c>
+      <c r="O32" s="15">
+        <v>504.14</v>
+      </c>
+      <c r="P32" s="15">
+        <v>495.48</v>
+      </c>
+      <c r="Q32" s="15">
+        <v>463.88</v>
+      </c>
+      <c r="R32" s="15">
+        <v>250.03</v>
+      </c>
+      <c r="S32" s="15">
+        <v>200.6</v>
+      </c>
+      <c r="T32" s="15">
+        <v>116.78</v>
+      </c>
+      <c r="U32" s="21">
+        <v>91.03</v>
+      </c>
+      <c r="V32" s="21">
+        <v>90.37</v>
+      </c>
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="13" t="s">
@@ -3215,8 +3240,8 @@
       <c r="V33" s="14"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="13" t="s">
-        <v>80</v>
+      <c r="A34" s="22" t="s">
+        <v>82</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -3264,7 +3289,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B35" s="21">
         <v>54.0</v>
@@ -3332,7 +3357,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B36" s="21">
         <v>13.0</v>
@@ -3360,7 +3385,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B37" s="21">
         <v>60.0</v>
@@ -3388,7 +3413,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B38" s="20">
         <v>-19.0</v>
@@ -3416,7 +3441,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" s="21">
         <v>32.0</v>
@@ -3484,7 +3509,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -3516,7 +3541,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B41" s="19">
         <v>-337.0</v>
@@ -3582,7 +3607,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B42" s="19">
         <v>-374.0</v>
@@ -3610,7 +3635,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -3642,7 +3667,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -3676,7 +3701,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
@@ -3706,7 +3731,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B46" s="17">
         <v>29700.0</v>
@@ -3774,7 +3799,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B47" s="20">
         <v>-1.0</v>
@@ -3814,7 +3839,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B48" s="18">
         <v>5665.0</v>
@@ -3876,13 +3901,13 @@
       <c r="U48" s="18">
         <v>264.7</v>
       </c>
-      <c r="V48" s="22">
+      <c r="V48" s="23">
         <v>91.48</v>
       </c>
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B49" s="14"/>
       <c r="C49" s="15">
@@ -3948,7 +3973,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B50" s="19">
         <v>-1402.0</v>
@@ -4000,7 +4025,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B51" s="19">
         <v>-765.0</v>
@@ -4068,7 +4093,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B52" s="19">
         <v>-150.0</v>
@@ -4106,7 +4131,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -4136,7 +4161,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B54" s="19">
         <v>-472.0</v>
@@ -4188,7 +4213,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B55" s="20">
         <v>-15.0</v>
@@ -4240,7 +4265,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -4274,7 +4299,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -4316,7 +4341,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B58" s="15">
         <v>760.0</v>
@@ -4368,7 +4393,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B59" s="15">
         <v>293.0</v>
@@ -4436,7 +4461,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B60" s="15">
         <v>453.0</v>
@@ -4504,7 +4529,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B61" s="21">
         <v>13.0</v>
@@ -4572,7 +4597,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B62" s="21">
         <v>1.0</v>
@@ -4602,7 +4627,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -4636,7 +4661,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B64" s="14"/>
       <c r="C64" s="14"/>
@@ -4666,21 +4691,21 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B65" s="23">
+        <v>113</v>
+      </c>
+      <c r="B65" s="24">
         <v>-642.0</v>
       </c>
-      <c r="C65" s="23">
+      <c r="C65" s="24">
         <v>-307.0</v>
       </c>
       <c r="D65" s="18">
         <v>187.0</v>
       </c>
-      <c r="E65" s="22">
+      <c r="E65" s="23">
         <v>44.0</v>
       </c>
-      <c r="F65" s="23">
+      <c r="F65" s="24">
         <v>-177.0</v>
       </c>
       <c r="G65" s="18">
@@ -4695,46 +4720,46 @@
       <c r="J65" s="18">
         <v>220.0</v>
       </c>
-      <c r="K65" s="24">
+      <c r="K65" s="25">
         <v>-61.0</v>
       </c>
-      <c r="L65" s="23">
+      <c r="L65" s="24">
         <v>-129.54</v>
       </c>
-      <c r="M65" s="24">
+      <c r="M65" s="25">
         <v>-75.79</v>
       </c>
-      <c r="N65" s="23">
+      <c r="N65" s="24">
         <v>-115.47</v>
       </c>
-      <c r="O65" s="23">
+      <c r="O65" s="24">
         <v>-145.23</v>
       </c>
-      <c r="P65" s="24">
+      <c r="P65" s="25">
         <v>-56.82</v>
       </c>
-      <c r="Q65" s="23">
+      <c r="Q65" s="24">
         <v>-172.64</v>
       </c>
-      <c r="R65" s="23">
+      <c r="R65" s="24">
         <v>-311.74</v>
       </c>
-      <c r="S65" s="24">
+      <c r="S65" s="25">
         <v>-62.85</v>
       </c>
-      <c r="T65" s="24">
+      <c r="T65" s="25">
         <v>-31.61</v>
       </c>
-      <c r="U65" s="24">
+      <c r="U65" s="25">
         <v>-32.52</v>
       </c>
-      <c r="V65" s="24">
+      <c r="V65" s="25">
         <v>-27.63</v>
       </c>
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B66" s="20">
         <v>-1.0</v>
@@ -4765,10 +4790,10 @@
         <v>0.0</v>
       </c>
       <c r="P66" s="14"/>
-      <c r="Q66" s="25">
+      <c r="Q66" s="26">
         <v>0.0</v>
       </c>
-      <c r="R66" s="25">
+      <c r="R66" s="26">
         <v>0.0</v>
       </c>
       <c r="S66" s="14"/>
@@ -4778,7 +4803,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B67" s="18">
         <v>5022.0</v>
@@ -4840,13 +4865,13 @@
       <c r="U67" s="18">
         <v>232.18</v>
       </c>
-      <c r="V67" s="22">
+      <c r="V67" s="23">
         <v>63.85</v>
       </c>
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B68" s="15">
         <v>133.0</v>
@@ -4914,7 +4939,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B69" s="19">
         <v>-797.0</v>
@@ -4944,7 +4969,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B70" s="15">
         <v>308.0</v>
@@ -5010,7 +5035,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B71" s="14"/>
       <c r="C71" s="14"/>
@@ -5052,7 +5077,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B72" s="19">
         <v>-128.0</v>
@@ -5102,7 +5127,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B73" s="15">
         <v>750.0</v>
@@ -5152,7 +5177,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B74" s="14"/>
       <c r="C74" s="14"/>
@@ -5196,7 +5221,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B75" s="18">
         <v>133.0</v>
@@ -5249,22 +5274,22 @@
       <c r="R75" s="18">
         <v>120.85</v>
       </c>
-      <c r="S75" s="22">
+      <c r="S75" s="23">
         <v>32.34</v>
       </c>
-      <c r="T75" s="22">
+      <c r="T75" s="23">
         <v>35.42</v>
       </c>
-      <c r="U75" s="24">
+      <c r="U75" s="25">
         <v>-13.29</v>
       </c>
-      <c r="V75" s="24">
+      <c r="V75" s="25">
         <v>-19.06</v>
       </c>
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="14"/>
@@ -5284,7 +5309,7 @@
       <c r="K76" s="14"/>
       <c r="L76" s="14"/>
       <c r="M76" s="14"/>
-      <c r="N76" s="25">
+      <c r="N76" s="26">
         <v>0.0</v>
       </c>
       <c r="O76" s="14"/>
@@ -5302,7 +5327,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B77" s="18">
         <v>4889.0</v>
@@ -5364,13 +5389,13 @@
       <c r="U77" s="18">
         <v>245.47</v>
       </c>
-      <c r="V77" s="22">
+      <c r="V77" s="23">
         <v>82.91</v>
       </c>
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B78" s="21">
         <v>1.0</v>
@@ -5398,7 +5423,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B79" s="18">
         <v>4890.0</v>
@@ -5460,13 +5485,13 @@
       <c r="U79" s="18">
         <v>245.47</v>
       </c>
-      <c r="V79" s="22">
+      <c r="V79" s="23">
         <v>82.91</v>
       </c>
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B80" s="14"/>
       <c r="C80" s="14"/>
@@ -5504,7 +5529,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B81" s="17"/>
       <c r="C81" s="17"/>
@@ -5519,10 +5544,10 @@
       <c r="L81" s="17">
         <v>0.0</v>
       </c>
-      <c r="M81" s="23">
+      <c r="M81" s="24">
         <v>-238.7</v>
       </c>
-      <c r="N81" s="22">
+      <c r="N81" s="23">
         <v>59.09</v>
       </c>
       <c r="O81" s="17"/>
@@ -5535,14 +5560,14 @@
       <c r="T81" s="18">
         <v>108.34</v>
       </c>
-      <c r="U81" s="22">
+      <c r="U81" s="23">
         <v>5.13</v>
       </c>
       <c r="V81" s="17"/>
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B82" s="15">
         <v>2144.0</v>
@@ -5610,12 +5635,12 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B83" s="18">
         <v>2144.0</v>
       </c>
-      <c r="C83" s="22">
+      <c r="C83" s="23">
         <v>52.0</v>
       </c>
       <c r="D83" s="18">
@@ -5660,25 +5685,25 @@
       <c r="Q83" s="18">
         <v>264.61</v>
       </c>
-      <c r="R83" s="22">
+      <c r="R83" s="23">
         <v>40.46</v>
       </c>
-      <c r="S83" s="22">
+      <c r="S83" s="23">
         <v>8.56</v>
       </c>
-      <c r="T83" s="22">
+      <c r="T83" s="23">
         <v>2.27</v>
       </c>
-      <c r="U83" s="22">
+      <c r="U83" s="23">
         <v>9.87</v>
       </c>
-      <c r="V83" s="22">
+      <c r="V83" s="23">
         <v>4.88</v>
       </c>
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B84" s="14"/>
       <c r="C84" s="14"/>
@@ -5695,10 +5720,10 @@
       <c r="N84" s="14"/>
       <c r="O84" s="14"/>
       <c r="P84" s="14"/>
-      <c r="Q84" s="25">
+      <c r="Q84" s="26">
         <v>0.0</v>
       </c>
-      <c r="R84" s="25">
+      <c r="R84" s="26">
         <v>0.0</v>
       </c>
       <c r="S84" s="14"/>
@@ -5708,7 +5733,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B85" s="18">
         <v>2746.0</v>
@@ -5770,13 +5795,13 @@
       <c r="U85" s="18">
         <v>240.74</v>
       </c>
-      <c r="V85" s="22">
+      <c r="V85" s="23">
         <v>78.03</v>
       </c>
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B86" s="14"/>
       <c r="C86" s="14"/>
@@ -5793,7 +5818,7 @@
       <c r="L86" s="14"/>
       <c r="M86" s="14"/>
       <c r="N86" s="14"/>
-      <c r="O86" s="25">
+      <c r="O86" s="26">
         <v>0.0</v>
       </c>
       <c r="P86" s="14"/>
@@ -5810,7 +5835,7 @@
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B87" s="18">
         <v>2746.0</v>
@@ -5872,13 +5897,13 @@
       <c r="U87" s="18">
         <v>235.6</v>
       </c>
-      <c r="V87" s="22">
+      <c r="V87" s="23">
         <v>78.03</v>
       </c>
     </row>
     <row r="88" ht="15.0" customHeight="1">
       <c r="A88" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B88" s="20">
         <v>-1.0</v>
@@ -5899,7 +5924,7 @@
       <c r="L88" s="14"/>
       <c r="M88" s="14"/>
       <c r="N88" s="14"/>
-      <c r="O88" s="25">
+      <c r="O88" s="26">
         <v>0.0</v>
       </c>
       <c r="P88" s="14"/>
@@ -5916,7 +5941,7 @@
     </row>
     <row r="89" ht="15.0" customHeight="1">
       <c r="A89" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B89" s="18">
         <v>2745.0</v>
@@ -5978,13 +6003,13 @@
       <c r="U89" s="18">
         <v>240.74</v>
       </c>
-      <c r="V89" s="22">
+      <c r="V89" s="23">
         <v>78.03</v>
       </c>
     </row>
     <row r="90" ht="15.0" customHeight="1">
       <c r="A90" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B90" s="15">
         <v>4890.0</v>
@@ -6026,7 +6051,7 @@
     </row>
     <row r="91" ht="15.0" customHeight="1">
       <c r="A91" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B91" s="15">
         <v>512.0</v>
@@ -6068,7 +6093,7 @@
     </row>
     <row r="92" ht="15.0" customHeight="1">
       <c r="A92" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B92" s="21">
         <v>2.0</v>
@@ -6110,7 +6135,7 @@
     </row>
     <row r="93" ht="15.0" customHeight="1">
       <c r="A93" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B93" s="20">
         <v>-24.0</v>
@@ -6152,7 +6177,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B94" s="20">
         <v>-9.0</v>
@@ -6194,7 +6219,7 @@
     </row>
     <row r="95" ht="15.0" customHeight="1">
       <c r="A95" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B95" s="14"/>
       <c r="C95" s="14"/>
@@ -6226,7 +6251,7 @@
     </row>
     <row r="96" ht="15.0" customHeight="1">
       <c r="A96" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B96" s="20">
         <v>-1.0</v>
@@ -6260,7 +6285,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B97" s="18">
         <v>480.0</v>
@@ -6271,19 +6296,19 @@
       <c r="D97" s="18">
         <v>442.0</v>
       </c>
-      <c r="E97" s="24">
+      <c r="E97" s="25">
         <v>-16.0</v>
       </c>
-      <c r="F97" s="23">
+      <c r="F97" s="24">
         <v>-174.0</v>
       </c>
-      <c r="G97" s="22">
+      <c r="G97" s="23">
         <v>96.0</v>
       </c>
       <c r="H97" s="18">
         <v>125.0</v>
       </c>
-      <c r="I97" s="22">
+      <c r="I97" s="23">
         <v>82.0</v>
       </c>
       <c r="J97" s="17"/>
@@ -6302,7 +6327,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B98" s="15">
         <v>2224.0</v>
@@ -6344,7 +6369,7 @@
     </row>
     <row r="99" ht="15.0" customHeight="1">
       <c r="A99" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B99" s="15">
         <v>3146.0</v>
@@ -6386,7 +6411,7 @@
     </row>
     <row r="100" ht="15.0" customHeight="1">
       <c r="A100" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B100" s="20">
         <v>-1.0</v>
@@ -6422,7 +6447,7 @@
     </row>
     <row r="101" ht="15.0" customHeight="1">
       <c r="A101" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B101" s="18">
         <v>5370.0</v>
@@ -6464,7 +6489,7 @@
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B102" s="15">
         <v>201.82</v>
@@ -6532,7 +6557,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B103" s="15">
         <v>201.82</v>
@@ -6600,7 +6625,7 @@
     </row>
     <row r="104" ht="15.0" customHeight="1">
       <c r="A104" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B104" s="15">
         <v>2746.0</v>
@@ -6668,7 +6693,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B105" s="21">
         <v>13.6</v>
@@ -6736,7 +6761,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B106" s="21">
         <v>13.6</v>
@@ -6804,7 +6829,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B107" s="21">
         <v>13.61</v>
@@ -6872,7 +6897,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B108" s="21">
         <v>13.61</v>
@@ -6940,7 +6965,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B109" s="15">
         <v>2745.0</v>
@@ -7044,7 +7069,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B111" s="14"/>
       <c r="C111" s="14"/>
@@ -7076,7 +7101,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B112" s="14"/>
       <c r="C112" s="14"/>
@@ -7106,7 +7131,7 @@
     </row>
     <row r="113" ht="15.0" customHeight="1">
       <c r="A113" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B113" s="14"/>
       <c r="C113" s="14"/>
@@ -7136,7 +7161,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B114" s="14"/>
       <c r="C114" s="14"/>
@@ -7166,7 +7191,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B115" s="14"/>
       <c r="C115" s="14"/>
@@ -7208,7 +7233,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B116" s="14"/>
       <c r="C116" s="14"/>
@@ -7240,7 +7265,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B117" s="21">
         <v>0.05</v>
@@ -7302,7 +7327,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B118" s="21">
         <v>0.01</v>
@@ -7332,7 +7357,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B119" s="14">
         <v>0.0</v>
@@ -7394,7 +7419,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B120" s="14"/>
       <c r="C120" s="14"/>
@@ -7448,7 +7473,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B121" s="21">
         <v>0.01</v>
@@ -7480,7 +7505,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B122" s="21">
         <v>0.03</v>
@@ -7542,7 +7567,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B123" s="14"/>
       <c r="C123" s="14"/>
@@ -7578,7 +7603,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B124" s="14"/>
       <c r="C124" s="14"/>
@@ -7608,7 +7633,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B125" s="21">
         <v>32.0</v>
@@ -7638,7 +7663,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B126" s="14"/>
       <c r="C126" s="14"/>
@@ -7684,7 +7709,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B127" s="21">
         <v>32.0</v>
@@ -7752,7 +7777,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B128" s="15">
         <v>2033.0</v>
@@ -7802,7 +7827,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B129" s="15">
         <v>2065.0</v>
@@ -7870,7 +7895,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B130" s="15">
         <v>150.0</v>
@@ -7902,7 +7927,7 @@
     </row>
     <row r="131" ht="15.0" customHeight="1">
       <c r="A131" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B131" s="14"/>
       <c r="C131" s="14"/>
@@ -7932,7 +7957,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B132" s="14"/>
       <c r="C132" s="14"/>
@@ -7962,7 +7987,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B133" s="20">
         <v>-74.0</v>
@@ -7992,7 +8017,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B134" s="15">
         <v>201.82</v>
@@ -8044,7 +8069,7 @@
     </row>
     <row r="135" ht="15.0" customHeight="1">
       <c r="A135" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B135" s="15">
         <v>201.82</v>
@@ -8096,7 +8121,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B136" s="21">
         <v>13.61</v>
@@ -8148,7 +8173,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B137" s="21">
         <v>13.6</v>
@@ -8200,7 +8225,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B138" s="21">
         <v>13.6</v>
@@ -8252,7 +8277,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B139" s="21">
         <v>13.61</v>
@@ -8304,7 +8329,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B140" s="15">
         <v>2745.0</v>
@@ -8356,7 +8381,7 @@
     </row>
     <row r="141" ht="15.0" customHeight="1">
       <c r="A141" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B141" s="15">
         <v>2745.0</v>
@@ -8408,7 +8433,7 @@
     </row>
     <row r="142" ht="15.0" customHeight="1">
       <c r="A142" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B142" s="21">
         <v>1.0</v>
@@ -8460,7 +8485,7 @@
     </row>
     <row r="143" ht="15.0" customHeight="1">
       <c r="A143" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B143" s="21">
         <v>1.0</v>
@@ -8512,7 +8537,7 @@
     </row>
     <row r="144" ht="15.0" customHeight="1">
       <c r="A144" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B144" s="15">
         <v>2746.0</v>
@@ -8564,7 +8589,7 @@
     </row>
     <row r="145" ht="15.0" customHeight="1">
       <c r="A145" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B145" s="15">
         <v>2746.0</v>
@@ -9491,7 +9516,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -9864,72 +9889,72 @@
         <v>43</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -10023,7 +10048,7 @@
     </row>
     <row r="19" ht="15.0" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B19" s="15">
         <v>3652.0</v>
@@ -10087,7 +10112,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B20" s="15">
         <v>964.0</v>
@@ -10149,7 +10174,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B21" s="15">
         <v>150.0</v>
@@ -10211,7 +10236,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B22" s="15">
         <v>2557.0</v>
@@ -10273,7 +10298,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B23" s="20">
         <v>-19.0</v>
@@ -10335,7 +10360,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -10371,7 +10396,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B25" s="14">
         <v>10049.0</v>
@@ -10435,7 +10460,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B26" s="15">
         <v>3501.0</v>
@@ -10489,7 +10514,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B27" s="15">
         <v>3525.0</v>
@@ -10551,7 +10576,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B28" s="20">
         <v>-24.0</v>
@@ -10613,7 +10638,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
@@ -10643,7 +10668,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B30" s="15">
         <v>1379.0</v>
@@ -10711,7 +10736,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B31" s="15">
         <v>302.0</v>
@@ -10767,7 +10792,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B32" s="21">
         <v>62.0</v>
@@ -10823,7 +10848,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B33" s="21">
         <v>35.0</v>
@@ -10873,7 +10898,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B34" s="15">
         <v>980.0</v>
@@ -10923,7 +10948,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -10955,7 +10980,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B36" s="15">
         <v>5719.0</v>
@@ -11023,7 +11048,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B37" s="15">
         <v>135.0</v>
@@ -11063,7 +11088,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B38" s="15">
         <v>5584.0</v>
@@ -11103,7 +11128,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -11139,7 +11164,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B40" s="21">
         <v>1.0</v>
@@ -11177,10 +11202,10 @@
         <v>1341.11</v>
       </c>
       <c r="Q40" s="14"/>
-      <c r="R40" s="25">
+      <c r="R40" s="26">
         <v>0.0</v>
       </c>
-      <c r="S40" s="25">
+      <c r="S40" s="26">
         <v>0.0</v>
       </c>
       <c r="T40" s="14"/>
@@ -11189,7 +11214,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="16" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B41" s="17">
         <v>24301.0</v>
@@ -11257,7 +11282,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
@@ -11285,7 +11310,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -11323,7 +11348,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B44" s="15">
         <v>2294.0</v>
@@ -11383,7 +11408,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B45" s="15">
         <v>2435.0</v>
@@ -11437,7 +11462,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B46" s="19">
         <v>-141.0</v>
@@ -11491,7 +11516,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="20">
@@ -11523,7 +11548,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B48" s="15">
         <v>9161.0</v>
@@ -11581,7 +11606,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B49" s="14">
         <v>10082.0</v>
@@ -11639,7 +11664,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B50" s="19">
         <v>-925.0</v>
@@ -11693,7 +11718,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B51" s="21">
         <v>4.0</v>
@@ -11735,7 +11760,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B52" s="21">
         <v>50.0</v>
@@ -11793,7 +11818,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="13" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B53" s="21">
         <v>50.0</v>
@@ -11849,7 +11874,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="13" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B54" s="14">
         <v>0.0</v>
@@ -11905,7 +11930,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -11933,7 +11958,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -11965,7 +11990,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B57" s="15">
         <v>2890.0</v>
@@ -12019,7 +12044,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B58" s="15">
         <v>6715.0</v>
@@ -12081,7 +12106,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B59" s="19">
         <v>-3825.0</v>
@@ -12135,7 +12160,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B60" s="14"/>
       <c r="C60" s="14"/>
@@ -12167,7 +12192,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
@@ -12197,7 +12222,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B62" s="14"/>
       <c r="C62" s="14"/>
@@ -12227,7 +12252,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -12257,7 +12282,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B64" s="14"/>
       <c r="C64" s="14"/>
@@ -12287,7 +12312,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B65" s="15">
         <v>9153.0</v>
@@ -12341,7 +12366,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B66" s="15">
         <v>648.0</v>
@@ -12395,7 +12420,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B67" s="15">
         <v>650.0</v>
@@ -12457,7 +12482,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B68" s="20">
         <v>-1.0</v>
@@ -12511,7 +12536,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B69" s="20">
         <v>-1.0</v>
@@ -12543,7 +12568,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B70" s="15">
         <v>617.0</v>
@@ -12597,7 +12622,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B71" s="15">
         <v>651.0</v>
@@ -12655,7 +12680,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B72" s="20">
         <v>-34.0</v>
@@ -12705,7 +12730,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
@@ -12739,7 +12764,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B74" s="15">
         <v>4619.0</v>
@@ -12793,7 +12818,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B75" s="15">
         <v>7418.0</v>
@@ -12855,7 +12880,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B76" s="19">
         <v>-2799.0</v>
@@ -12909,7 +12934,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B77" s="14"/>
       <c r="C77" s="14"/>
@@ -12930,7 +12955,7 @@
       <c r="L77" s="21">
         <v>1.0</v>
       </c>
-      <c r="M77" s="25">
+      <c r="M77" s="26">
         <v>0.0</v>
       </c>
       <c r="N77" s="14"/>
@@ -12945,7 +12970,7 @@
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B78" s="15">
         <v>3267.0</v>
@@ -12999,7 +13024,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B79" s="15">
         <v>9942.0</v>
@@ -13049,7 +13074,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B80" s="19">
         <v>-6675.0</v>
@@ -13103,7 +13128,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B81" s="14"/>
       <c r="C81" s="14"/>
@@ -13131,7 +13156,7 @@
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B82" s="14"/>
       <c r="C82" s="14"/>
@@ -13159,7 +13184,7 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B83" s="21">
         <v>2.0</v>
@@ -13190,7 +13215,7 @@
       <c r="L83" s="21">
         <v>1.0</v>
       </c>
-      <c r="M83" s="25">
+      <c r="M83" s="26">
         <v>0.0</v>
       </c>
       <c r="N83" s="14"/>
@@ -13243,7 +13268,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B85" s="14"/>
       <c r="C85" s="14"/>
@@ -13261,7 +13286,7 @@
       <c r="O85" s="15">
         <v>3760.06</v>
       </c>
-      <c r="P85" s="26">
+      <c r="P85" s="27">
         <v>3500.0</v>
       </c>
       <c r="Q85" s="15">
@@ -13283,7 +13308,7 @@
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B86" s="15">
         <v>3500.0</v>
@@ -13321,7 +13346,7 @@
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B87" s="15">
         <v>7071.0</v>
@@ -13359,7 +13384,7 @@
     </row>
     <row r="88" ht="15.0" customHeight="1">
       <c r="A88" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B88" s="19">
         <v>-3571.0</v>
@@ -13397,7 +13422,7 @@
     </row>
     <row r="89" ht="15.0" customHeight="1">
       <c r="A89" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B89" s="15">
         <v>3803.0</v>
@@ -13465,7 +13490,7 @@
     </row>
     <row r="90" ht="15.0" customHeight="1">
       <c r="A90" s="13" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B90" s="21">
         <v>40.0</v>
@@ -13533,7 +13558,7 @@
     </row>
     <row r="91" ht="15.0" customHeight="1">
       <c r="A91" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B91" s="15">
         <v>245.0</v>
@@ -13593,7 +13618,7 @@
     </row>
     <row r="92" ht="15.0" customHeight="1">
       <c r="A92" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B92" s="14"/>
       <c r="C92" s="14"/>
@@ -13637,7 +13662,7 @@
     </row>
     <row r="93" ht="15.0" customHeight="1">
       <c r="A93" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B93" s="14"/>
       <c r="C93" s="14"/>
@@ -13681,7 +13706,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B94" s="15">
         <v>199.0</v>
@@ -13741,7 +13766,7 @@
     </row>
     <row r="95" ht="15.0" customHeight="1">
       <c r="A95" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B95" s="14"/>
       <c r="C95" s="14"/>
@@ -13771,7 +13796,7 @@
     </row>
     <row r="96" ht="15.0" customHeight="1">
       <c r="A96" s="13" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B96" s="14"/>
       <c r="C96" s="14"/>
@@ -13801,7 +13826,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B97" s="14"/>
       <c r="C97" s="14"/>
@@ -13831,7 +13856,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B98" s="14"/>
       <c r="C98" s="14"/>
@@ -13865,7 +13890,7 @@
     </row>
     <row r="99" ht="15.0" customHeight="1">
       <c r="A99" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B99" s="20">
         <v>-1.0</v>
@@ -13887,7 +13912,7 @@
       <c r="K99" s="14"/>
       <c r="L99" s="14"/>
       <c r="M99" s="14"/>
-      <c r="N99" s="25">
+      <c r="N99" s="26">
         <v>0.0</v>
       </c>
       <c r="O99" s="14"/>
@@ -13903,7 +13928,7 @@
     </row>
     <row r="100" ht="15.0" customHeight="1">
       <c r="A100" s="16" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B100" s="17">
         <v>31334.0</v>
@@ -13971,7 +13996,7 @@
     </row>
     <row r="101" ht="15.0" customHeight="1">
       <c r="A101" s="13" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B101" s="14"/>
       <c r="C101" s="21">
@@ -13992,7 +14017,7 @@
       </c>
       <c r="M101" s="14"/>
       <c r="N101" s="14"/>
-      <c r="O101" s="25">
+      <c r="O101" s="26">
         <v>0.0</v>
       </c>
       <c r="P101" s="14"/>
@@ -14011,7 +14036,7 @@
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="16" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B102" s="17">
         <v>55635.0</v>
@@ -14079,7 +14104,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B103" s="14"/>
       <c r="C103" s="14"/>
@@ -14122,8 +14147,8 @@
       <c r="V103" s="14"/>
     </row>
     <row r="104" ht="15.0" customHeight="1">
-      <c r="A104" s="27" t="s">
-        <v>272</v>
+      <c r="A104" s="22" t="s">
+        <v>273</v>
       </c>
       <c r="B104" s="14"/>
       <c r="C104" s="14"/>
@@ -14181,7 +14206,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B105" s="14"/>
       <c r="C105" s="14"/>
@@ -14198,7 +14223,7 @@
         <v>-1.0</v>
       </c>
       <c r="L105" s="14"/>
-      <c r="M105" s="25">
+      <c r="M105" s="26">
         <v>0.0</v>
       </c>
       <c r="N105" s="14"/>
@@ -14215,7 +14240,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B106" s="15">
         <v>288.0</v>
@@ -14253,7 +14278,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B107" s="15">
         <v>417.0</v>
@@ -14310,8 +14335,8 @@
       <c r="V107" s="14"/>
     </row>
     <row r="108" ht="15.0" customHeight="1">
-      <c r="A108" s="27" t="s">
-        <v>276</v>
+      <c r="A108" s="22" t="s">
+        <v>277</v>
       </c>
       <c r="B108" s="15">
         <v>3927.0</v>
@@ -14341,7 +14366,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B109" s="15">
         <v>2348.0</v>
@@ -14403,7 +14428,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="13" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B110" s="15">
         <v>1579.0</v>
@@ -14439,7 +14464,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B111" s="14"/>
       <c r="C111" s="20">
@@ -14467,7 +14492,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B112" s="14"/>
       <c r="C112" s="14"/>
@@ -14517,7 +14542,7 @@
     </row>
     <row r="113" ht="15.0" customHeight="1">
       <c r="A113" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B113" s="15">
         <v>2600.0</v>
@@ -14585,7 +14610,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B114" s="15">
         <v>2169.0</v>
@@ -14651,7 +14676,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B115" s="15">
         <v>613.0</v>
@@ -14701,7 +14726,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B116" s="15">
         <v>671.0</v>
@@ -14751,7 +14776,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B117" s="15">
         <v>503.0</v>
@@ -14801,7 +14826,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B118" s="15">
         <v>112.0</v>
@@ -14851,7 +14876,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="13" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B119" s="21">
         <v>23.0</v>
@@ -14901,7 +14926,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="13" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B120" s="21">
         <v>24.0</v>
@@ -14933,7 +14958,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B121" s="15">
         <v>223.0</v>
@@ -14983,7 +15008,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="13" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B122" s="15">
         <v>211.0</v>
@@ -15049,7 +15074,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B123" s="14"/>
       <c r="C123" s="14"/>
@@ -15083,7 +15108,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B124" s="20">
         <v>-1.0</v>
@@ -15110,7 +15135,7 @@
       <c r="P124" s="15">
         <v>771.47</v>
       </c>
-      <c r="Q124" s="25">
+      <c r="Q124" s="26">
         <v>0.0</v>
       </c>
       <c r="R124" s="14">
@@ -15123,7 +15148,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="16" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B125" s="18">
         <v>9611.0</v>
@@ -15191,7 +15216,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B126" s="14"/>
       <c r="C126" s="14"/>
@@ -15235,7 +15260,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B127" s="15">
         <v>918.0</v>
@@ -15291,7 +15316,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B128" s="15">
         <v>1769.0</v>
@@ -15329,7 +15354,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B129" s="15">
         <v>8588.0</v>
@@ -15393,7 +15418,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="13" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B130" s="15">
         <v>5061.0</v>
@@ -15425,7 +15450,7 @@
     </row>
     <row r="131" ht="15.0" customHeight="1">
       <c r="A131" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B131" s="14"/>
       <c r="C131" s="14"/>
@@ -15487,7 +15512,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="13" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B132" s="21">
         <v>6.0</v>
@@ -15555,7 +15580,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B133" s="21">
         <v>15.0</v>
@@ -15613,7 +15638,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="13" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B134" s="14"/>
       <c r="C134" s="14"/>
@@ -15641,7 +15666,7 @@
       <c r="Q134" s="14">
         <v>0.0</v>
       </c>
-      <c r="R134" s="25">
+      <c r="R134" s="26">
         <v>0.0</v>
       </c>
       <c r="S134" s="14"/>
@@ -15651,7 +15676,7 @@
     </row>
     <row r="135" ht="15.0" customHeight="1">
       <c r="A135" s="16" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B135" s="17">
         <v>16357.0</v>
@@ -15719,7 +15744,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="13" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B136" s="14"/>
       <c r="C136" s="14"/>
@@ -15751,7 +15776,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="16" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B137" s="17">
         <v>25968.0</v>
@@ -15819,7 +15844,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="13" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B138" s="15">
         <v>101.0</v>
@@ -15887,7 +15912,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B139" s="15">
         <v>3714.0</v>
@@ -15955,7 +15980,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="13" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B140" s="14">
         <v>13281.0</v>
@@ -16023,7 +16048,7 @@
     </row>
     <row r="141" ht="15.0" customHeight="1">
       <c r="A141" s="13" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B141" s="15">
         <v>2351.0</v>
@@ -16075,7 +16100,7 @@
     </row>
     <row r="142" ht="15.0" customHeight="1">
       <c r="A142" s="13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B142" s="21">
         <v>95.0</v>
@@ -16127,7 +16152,7 @@
     </row>
     <row r="143" ht="15.0" customHeight="1">
       <c r="A143" s="13" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B143" s="14">
         <v>10834.0</v>
@@ -16179,7 +16204,7 @@
     </row>
     <row r="144" ht="15.0" customHeight="1">
       <c r="A144" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B144" s="21">
         <v>1.0</v>
@@ -16200,7 +16225,7 @@
       </c>
       <c r="K144" s="14"/>
       <c r="L144" s="14"/>
-      <c r="M144" s="25">
+      <c r="M144" s="26">
         <v>0.0</v>
       </c>
       <c r="N144" s="14"/>
@@ -16215,7 +16240,7 @@
     </row>
     <row r="145" ht="15.0" customHeight="1">
       <c r="A145" s="13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B145" s="20">
         <v>-18.0</v>
@@ -16267,7 +16292,7 @@
     </row>
     <row r="146" ht="15.0" customHeight="1">
       <c r="A146" s="13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B146" s="14"/>
       <c r="C146" s="14"/>
@@ -16288,7 +16313,7 @@
       <c r="L146" s="14"/>
       <c r="M146" s="14"/>
       <c r="N146" s="14"/>
-      <c r="O146" s="25">
+      <c r="O146" s="26">
         <v>0.0</v>
       </c>
       <c r="P146" s="14"/>
@@ -16301,7 +16326,7 @@
     </row>
     <row r="147" ht="15.0" customHeight="1">
       <c r="A147" s="16" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B147" s="17">
         <v>17078.0</v>
@@ -16369,7 +16394,7 @@
     </row>
     <row r="148" ht="15.0" customHeight="1">
       <c r="A148" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B148" s="14">
         <v>12590.0</v>
@@ -16437,7 +16462,7 @@
     </row>
     <row r="149" ht="15.0" customHeight="1">
       <c r="A149" s="16" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B149" s="17">
         <v>12590.0</v>
@@ -16489,7 +16514,7 @@
     </row>
     <row r="150" ht="15.0" customHeight="1">
       <c r="A150" s="16" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B150" s="17">
         <v>29668.0</v>
@@ -16557,7 +16582,7 @@
     </row>
     <row r="151" ht="15.0" customHeight="1">
       <c r="A151" s="13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B151" s="20">
         <v>-1.0</v>
@@ -16582,7 +16607,7 @@
       <c r="P151" s="14"/>
       <c r="Q151" s="14"/>
       <c r="R151" s="14"/>
-      <c r="S151" s="25">
+      <c r="S151" s="26">
         <v>0.0</v>
       </c>
       <c r="T151" s="14"/>
@@ -16591,7 +16616,7 @@
     </row>
     <row r="152" ht="15.0" customHeight="1">
       <c r="A152" s="16" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B152" s="17">
         <v>55635.0</v>
@@ -16659,7 +16684,7 @@
     </row>
     <row r="153" ht="15.0" customHeight="1">
       <c r="A153" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B153" s="15">
         <v>201.82</v>
@@ -16727,7 +16752,7 @@
     </row>
     <row r="154" ht="15.0" customHeight="1">
       <c r="A154" s="13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B154" s="21">
         <v>0.89</v>
@@ -16795,7 +16820,7 @@
     </row>
     <row r="155" ht="15.0" customHeight="1">
       <c r="A155" s="13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B155" s="15">
         <v>202.72</v>
@@ -16863,7 +16888,7 @@
     </row>
     <row r="156" ht="15.0" customHeight="1">
       <c r="A156" s="13" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B156" s="14"/>
       <c r="C156" s="14"/>
@@ -16895,7 +16920,7 @@
     </row>
     <row r="157" ht="15.0" customHeight="1">
       <c r="A157" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B157" s="14"/>
       <c r="C157" s="14"/>
@@ -16923,7 +16948,7 @@
     </row>
     <row r="158" ht="15.0" customHeight="1">
       <c r="A158" s="13" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B158" s="14"/>
       <c r="C158" s="14"/>
@@ -16951,7 +16976,7 @@
     </row>
     <row r="159" ht="15.0" customHeight="1">
       <c r="A159" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B159" s="14"/>
       <c r="C159" s="14"/>
@@ -16979,7 +17004,7 @@
     </row>
     <row r="160" ht="15.0" customHeight="1">
       <c r="A160" s="13" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B160" s="14">
         <v>14450.0</v>
@@ -17031,7 +17056,7 @@
     </row>
     <row r="161" ht="15.0" customHeight="1">
       <c r="A161" s="13" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B161" s="15">
         <v>4442.0</v>
@@ -17083,7 +17108,7 @@
     </row>
     <row r="162" ht="15.0" customHeight="1">
       <c r="A162" s="13" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B162" s="15">
         <v>3212.0</v>
@@ -17135,7 +17160,7 @@
     </row>
     <row r="163" ht="15.0" customHeight="1">
       <c r="A163" s="13" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B163" s="15">
         <v>3769.0</v>
@@ -17187,7 +17212,7 @@
     </row>
     <row r="164" ht="15.0" customHeight="1">
       <c r="A164" s="13" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B164" s="14"/>
       <c r="C164" s="14"/>
@@ -17215,7 +17240,7 @@
     </row>
     <row r="165" ht="15.0" customHeight="1">
       <c r="A165" s="13" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B165" s="15">
         <v>3027.0</v>
@@ -17267,7 +17292,7 @@
     </row>
     <row r="166" ht="15.0" customHeight="1">
       <c r="A166" s="13" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B166" s="14"/>
       <c r="C166" s="14"/>
@@ -17297,7 +17322,7 @@
     </row>
     <row r="167" ht="15.0" customHeight="1">
       <c r="A167" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B167" s="14"/>
       <c r="C167" s="14"/>
@@ -17343,7 +17368,7 @@
     </row>
     <row r="168" ht="15.0" customHeight="1">
       <c r="A168" s="13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B168" s="14"/>
       <c r="C168" s="14"/>
@@ -17389,7 +17414,7 @@
     </row>
     <row r="169" ht="15.0" customHeight="1">
       <c r="A169" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B169" s="15">
         <v>3815.0</v>
@@ -17441,7 +17466,7 @@
     </row>
     <row r="170" ht="15.0" customHeight="1">
       <c r="A170" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B170" s="15">
         <v>865.0</v>
@@ -17493,7 +17518,7 @@
     </row>
     <row r="171" ht="15.0" customHeight="1">
       <c r="A171" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B171" s="15">
         <v>1404.0</v>
@@ -17531,7 +17556,7 @@
     </row>
     <row r="172" ht="15.0" customHeight="1">
       <c r="A172" s="13" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B172" s="15">
         <v>799.0</v>
@@ -17583,7 +17608,7 @@
     </row>
     <row r="173" ht="15.0" customHeight="1">
       <c r="A173" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B173" s="15">
         <v>748.0</v>
@@ -17635,7 +17660,7 @@
     </row>
     <row r="174" ht="15.0" customHeight="1">
       <c r="A174" s="13" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B174" s="14"/>
       <c r="C174" s="14"/>
@@ -17669,7 +17694,7 @@
     </row>
     <row r="175" ht="15.0" customHeight="1">
       <c r="A175" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B175" s="20">
         <v>-1.0</v>
@@ -17697,7 +17722,7 @@
     </row>
     <row r="176" ht="15.0" customHeight="1">
       <c r="A176" s="13" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B176" s="14"/>
       <c r="C176" s="14"/>
@@ -17729,7 +17754,7 @@
     </row>
     <row r="177" ht="15.0" customHeight="1">
       <c r="A177" s="13" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B177" s="14"/>
       <c r="C177" s="14"/>
@@ -17761,7 +17786,7 @@
     </row>
     <row r="178" ht="15.0" customHeight="1">
       <c r="A178" s="13" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B178" s="15">
         <v>8924.0</v>
@@ -17791,7 +17816,7 @@
     </row>
     <row r="179" ht="15.0" customHeight="1">
       <c r="A179" s="13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B179" s="15">
         <v>201.82</v>
@@ -17859,7 +17884,7 @@
     </row>
     <row r="180" ht="15.0" customHeight="1">
       <c r="A180" s="13" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B180" s="21">
         <v>0.89</v>
@@ -17927,7 +17952,7 @@
     </row>
     <row r="181" ht="15.0" customHeight="1">
       <c r="A181" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B181" s="21">
         <v>1.0</v>
@@ -17995,7 +18020,7 @@
     </row>
     <row r="182" ht="15.0" customHeight="1">
       <c r="A182" s="13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B182" s="15">
         <v>202.72</v>
@@ -18063,7 +18088,7 @@
     </row>
     <row r="183" ht="15.0" customHeight="1">
       <c r="A183" s="13" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B183" s="15">
         <v>7320.0</v>
@@ -18125,7 +18150,7 @@
     </row>
     <row r="184" ht="15.0" customHeight="1">
       <c r="A184" s="13" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B184" s="14"/>
       <c r="C184" s="14"/>
@@ -18171,7 +18196,7 @@
     </row>
     <row r="185" ht="15.0" customHeight="1">
       <c r="A185" s="13" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B185" s="14"/>
       <c r="C185" s="14"/>
@@ -18217,7 +18242,7 @@
     </row>
     <row r="186" ht="15.0" customHeight="1">
       <c r="A186" s="13" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B186" s="14"/>
       <c r="C186" s="14"/>
@@ -18263,7 +18288,7 @@
     </row>
     <row r="187" ht="15.0" customHeight="1">
       <c r="A187" s="13" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B187" s="14"/>
       <c r="C187" s="14"/>
@@ -18309,7 +18334,7 @@
     </row>
     <row r="188" ht="15.0" customHeight="1">
       <c r="A188" s="13" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B188" s="14"/>
       <c r="C188" s="14"/>
@@ -18337,7 +18362,7 @@
     </row>
     <row r="189" ht="15.0" customHeight="1">
       <c r="A189" s="13" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B189" s="15">
         <v>9733.0</v>
@@ -19228,7 +19253,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -19601,72 +19626,72 @@
         <v>43</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -19760,7 +19785,7 @@
     </row>
     <row r="19" ht="15.0" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B19" s="15">
         <v>5022.0</v>
@@ -19828,7 +19853,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B20" s="19">
         <v>-1337.0</v>
@@ -19896,7 +19921,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B21" s="15">
         <v>2065.0</v>
@@ -19964,7 +19989,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B22" s="21">
         <v>54.0</v>
@@ -20030,7 +20055,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B23" s="19">
         <v>-374.0</v>
@@ -20098,7 +20123,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B24" s="15">
         <v>915.0</v>
@@ -20164,7 +20189,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B25" s="19">
         <v>-293.0</v>
@@ -20226,7 +20251,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B26" s="19">
         <v>-337.0</v>
@@ -20290,7 +20315,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B27" s="19">
         <v>-1522.0</v>
@@ -20358,7 +20383,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B28" s="19">
         <v>-514.0</v>
@@ -20426,7 +20451,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B29" s="20">
         <v>-91.0</v>
@@ -20494,7 +20519,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -20528,7 +20553,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -20556,7 +20581,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -20600,7 +20625,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B33" s="20">
         <v>-1.0</v>
@@ -20666,7 +20691,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B34" s="19">
         <v>-1277.0</v>
@@ -20696,7 +20721,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B35" s="20">
         <v>-10.0</v>
@@ -20754,7 +20779,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B36" s="21">
         <v>1.0</v>
@@ -20810,7 +20835,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B37" s="15">
         <v>600.0</v>
@@ -20870,7 +20895,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
@@ -20920,7 +20945,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -20952,7 +20977,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -20986,7 +21011,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
@@ -21020,7 +21045,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B42" s="21">
         <v>2.0</v>
@@ -21062,7 +21087,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="13" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -21092,7 +21117,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -21122,7 +21147,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="16" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B45" s="18">
         <v>2903.0</v>
@@ -21190,7 +21215,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B46" s="15">
         <v>110.0</v>
@@ -21258,7 +21283,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B47" s="15">
         <v>1955.0</v>
@@ -21290,7 +21315,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="13" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B48" s="19">
         <v>-2280.0</v>
@@ -21358,7 +21383,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B49" s="20">
         <v>-50.0</v>
@@ -21426,7 +21451,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B50" s="15">
         <v>221.0</v>
@@ -21490,7 +21515,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="13" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B51" s="15">
         <v>293.0</v>
@@ -21544,7 +21569,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="13" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B52" s="20">
         <v>-54.0</v>
@@ -21576,7 +21601,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="13" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -21632,7 +21657,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="13" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -21684,7 +21709,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="13" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B55" s="20">
         <v>-14.0</v>
@@ -21738,7 +21763,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="13" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -21788,7 +21813,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -21822,7 +21847,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="13" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -21852,7 +21877,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="13" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
@@ -21882,7 +21907,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="13" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B60" s="14"/>
       <c r="C60" s="21">
@@ -21926,75 +21951,75 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="16" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B61" s="18">
         <v>181.0</v>
       </c>
-      <c r="C61" s="23">
+      <c r="C61" s="24">
         <v>-1520.0</v>
       </c>
-      <c r="D61" s="23">
+      <c r="D61" s="24">
         <v>-1675.0</v>
       </c>
-      <c r="E61" s="23">
+      <c r="E61" s="24">
         <v>-1650.0</v>
       </c>
-      <c r="F61" s="23">
+      <c r="F61" s="24">
         <v>-1403.0</v>
       </c>
-      <c r="G61" s="23">
+      <c r="G61" s="24">
         <v>-1059.0</v>
       </c>
-      <c r="H61" s="23">
+      <c r="H61" s="24">
         <v>-1606.0</v>
       </c>
-      <c r="I61" s="23">
+      <c r="I61" s="24">
         <v>-1556.0</v>
       </c>
-      <c r="J61" s="23">
+      <c r="J61" s="24">
         <v>-3850.0</v>
       </c>
-      <c r="K61" s="23">
+      <c r="K61" s="24">
         <v>-878.0</v>
       </c>
       <c r="L61" s="18">
         <v>374.6</v>
       </c>
-      <c r="M61" s="23">
+      <c r="M61" s="24">
         <v>-1845.56</v>
       </c>
-      <c r="N61" s="23">
+      <c r="N61" s="24">
         <v>-679.96</v>
       </c>
-      <c r="O61" s="23">
+      <c r="O61" s="24">
         <v>-773.43</v>
       </c>
-      <c r="P61" s="23">
+      <c r="P61" s="24">
         <v>-520.2</v>
       </c>
       <c r="Q61" s="18">
         <v>224.9</v>
       </c>
-      <c r="R61" s="23">
+      <c r="R61" s="24">
         <v>-1448.19</v>
       </c>
-      <c r="S61" s="23">
+      <c r="S61" s="24">
         <v>-2195.46</v>
       </c>
-      <c r="T61" s="23">
+      <c r="T61" s="24">
         <v>-996.88</v>
       </c>
-      <c r="U61" s="23">
+      <c r="U61" s="24">
         <v>-162.83</v>
       </c>
-      <c r="V61" s="23">
+      <c r="V61" s="24">
         <v>-128.74</v>
       </c>
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="13" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B62" s="15">
         <v>2238.0</v>
@@ -22062,7 +22087,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="13" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B63" s="19">
         <v>-1582.0</v>
@@ -22130,7 +22155,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="13" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B64" s="14">
         <v>0.0</v>
@@ -22190,7 +22215,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="13" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B65" s="19">
         <v>-923.0</v>
@@ -22256,7 +22281,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="13" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B66" s="19">
         <v>-908.0</v>
@@ -22320,7 +22345,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="13" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B67" s="19">
         <v>-1788.0</v>
@@ -22366,7 +22391,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="13" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B68" s="15">
         <v>106.0</v>
@@ -22404,7 +22429,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="13" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B69" s="14"/>
       <c r="C69" s="14"/>
@@ -22452,7 +22477,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B70" s="14"/>
       <c r="C70" s="14"/>
@@ -22490,7 +22515,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="13" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B71" s="14"/>
       <c r="C71" s="14"/>
@@ -22524,7 +22549,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="13" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B72" s="14"/>
       <c r="C72" s="14"/>
@@ -22558,7 +22583,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="13" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
@@ -22596,7 +22621,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B74" s="14"/>
       <c r="C74" s="14"/>
@@ -22628,7 +22653,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="13" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B75" s="14"/>
       <c r="C75" s="14"/>
@@ -22656,7 +22681,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="13" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="21">
@@ -22692,54 +22717,54 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="16" t="s">
-        <v>409</v>
-      </c>
-      <c r="B77" s="23">
+        <v>410</v>
+      </c>
+      <c r="B77" s="24">
         <v>-2857.0</v>
       </c>
-      <c r="C77" s="23">
+      <c r="C77" s="24">
         <v>-551.0</v>
       </c>
-      <c r="D77" s="23">
+      <c r="D77" s="24">
         <v>-2547.0</v>
       </c>
-      <c r="E77" s="23">
+      <c r="E77" s="24">
         <v>-2128.0</v>
       </c>
-      <c r="F77" s="23">
+      <c r="F77" s="24">
         <v>-1326.0</v>
       </c>
-      <c r="G77" s="23">
+      <c r="G77" s="24">
         <v>-2256.0</v>
       </c>
-      <c r="H77" s="23">
+      <c r="H77" s="24">
         <v>-2253.0</v>
       </c>
-      <c r="I77" s="23">
+      <c r="I77" s="24">
         <v>-1326.0</v>
       </c>
       <c r="J77" s="18">
         <v>1827.0</v>
       </c>
-      <c r="K77" s="24">
+      <c r="K77" s="25">
         <v>-79.0</v>
       </c>
-      <c r="L77" s="23">
+      <c r="L77" s="24">
         <v>-1451.56</v>
       </c>
-      <c r="M77" s="23">
+      <c r="M77" s="24">
         <v>-396.42</v>
       </c>
-      <c r="N77" s="23">
+      <c r="N77" s="24">
         <v>-371.82</v>
       </c>
-      <c r="O77" s="23">
+      <c r="O77" s="24">
         <v>-688.73</v>
       </c>
-      <c r="P77" s="23">
+      <c r="P77" s="24">
         <v>-400.16</v>
       </c>
-      <c r="Q77" s="23">
+      <c r="Q77" s="24">
         <v>-907.88</v>
       </c>
       <c r="R77" s="18">
@@ -22754,13 +22779,13 @@
       <c r="U77" s="18">
         <v>131.64</v>
       </c>
-      <c r="V77" s="24">
+      <c r="V77" s="25">
         <v>-67.09</v>
       </c>
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="13" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B78" s="21">
         <v>17.0</v>
@@ -22828,7 +22853,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="13" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B79" s="15">
         <v>5475.0</v>
@@ -22896,7 +22921,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="13" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B80" s="15">
         <v>5719.0</v>
@@ -22964,7 +22989,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="13" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B81" s="15">
         <v>227.0</v>
@@ -23016,7 +23041,7 @@
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="16" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B82" s="18">
         <v>244.0</v>
@@ -23024,7 +23049,7 @@
       <c r="C82" s="18">
         <v>1135.0</v>
       </c>
-      <c r="D82" s="23">
+      <c r="D82" s="24">
         <v>-989.0</v>
       </c>
       <c r="E82" s="18">
@@ -23033,10 +23058,10 @@
       <c r="F82" s="18">
         <v>212.0</v>
       </c>
-      <c r="G82" s="23">
+      <c r="G82" s="24">
         <v>-142.0</v>
       </c>
-      <c r="H82" s="23">
+      <c r="H82" s="24">
         <v>-682.0</v>
       </c>
       <c r="I82" s="18">
@@ -23051,13 +23076,13 @@
       <c r="L82" s="18">
         <v>754.83</v>
       </c>
-      <c r="M82" s="23">
+      <c r="M82" s="24">
         <v>-725.37</v>
       </c>
-      <c r="N82" s="23">
+      <c r="N82" s="24">
         <v>-164.95</v>
       </c>
-      <c r="O82" s="23">
+      <c r="O82" s="24">
         <v>-427.62</v>
       </c>
       <c r="P82" s="18">
@@ -23066,10 +23091,10 @@
       <c r="Q82" s="18">
         <v>980.08</v>
       </c>
-      <c r="R82" s="23">
+      <c r="R82" s="24">
         <v>-397.37</v>
       </c>
-      <c r="S82" s="23">
+      <c r="S82" s="24">
         <v>-370.58</v>
       </c>
       <c r="T82" s="18">
@@ -23078,13 +23103,13 @@
       <c r="U82" s="18">
         <v>103.86</v>
       </c>
-      <c r="V82" s="24">
+      <c r="V82" s="25">
         <v>-52.86</v>
       </c>
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="13" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B83" s="14"/>
       <c r="C83" s="14"/>
@@ -23118,7 +23143,7 @@
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="13" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B84" s="14"/>
       <c r="C84" s="14"/>
@@ -24088,7 +24113,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -24526,7 +24551,7 @@
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -24620,7 +24645,7 @@
     </row>
     <row r="19" ht="15.0" customHeight="1">
       <c r="A19" s="28" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B19" s="29"/>
       <c r="C19" s="29"/>
@@ -24646,7 +24671,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="30" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B20" s="31">
         <v>42738.76</v>
@@ -24710,7 +24735,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="30" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B21" s="31">
         <v>38083.61</v>
@@ -24766,7 +24791,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="28" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B22" s="29"/>
       <c r="C22" s="29"/>
@@ -24792,7 +24817,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="30" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B23" s="31">
         <v>19825.76</v>
@@ -24856,7 +24881,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="30" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B24" s="31">
         <v>18427.01</v>
@@ -24912,7 +24937,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="28" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B25" s="29"/>
       <c r="C25" s="29"/>
@@ -24938,7 +24963,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="30" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B26" s="33">
         <v>97.8</v>
@@ -25002,7 +25027,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="30" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B27" s="33">
         <v>90.9</v>
@@ -25058,7 +25083,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="28" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -25084,7 +25109,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="30" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B29" s="34">
         <v>1.08</v>
@@ -25148,7 +25173,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="30" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B30" s="34">
         <v>7.18</v>
@@ -25204,7 +25229,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="28" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B31" s="29"/>
       <c r="C31" s="29"/>
@@ -25230,7 +25255,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="30" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B32" s="34">
         <v>3.59</v>
@@ -25294,7 +25319,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="30" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B33" s="34">
         <v>3.52</v>
@@ -25350,7 +25375,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="30" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B34" s="34">
         <v>4.6</v>
@@ -25414,7 +25439,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="30" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B35" s="34">
         <v>4.51</v>
@@ -25470,7 +25495,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="28" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29"/>
@@ -25496,7 +25521,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="30" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B37" s="33">
         <v>1.16</v>
@@ -25560,7 +25585,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="30" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B38" s="33">
         <v>1.26</v>
@@ -25616,7 +25641,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="28" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B39" s="29"/>
       <c r="C39" s="29"/>
@@ -25642,7 +25667,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="30" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B40" s="33">
         <v>3.54</v>
@@ -25698,7 +25723,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="30" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B41" s="33">
         <v>6.46</v>
@@ -25746,7 +25771,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="28" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B42" s="29"/>
       <c r="C42" s="29"/>
@@ -25772,7 +25797,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="30" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B43" s="33">
         <v>0.56</v>
@@ -25836,7 +25861,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="30" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B44" s="33">
         <v>0.61</v>
@@ -25892,7 +25917,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="28" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B45" s="29"/>
       <c r="C45" s="29"/>
@@ -25918,7 +25943,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="30" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B46" s="33">
         <v>92.24</v>
@@ -25976,7 +26001,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="30" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B47" s="33">
         <v>13.93</v>
@@ -26032,7 +26057,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="28" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B48" s="29"/>
       <c r="C48" s="29"/>
@@ -26058,7 +26083,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="30" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B49" s="33">
         <v>2.84</v>
@@ -26122,7 +26147,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="30" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B50" s="33">
         <v>4.06</v>
@@ -26178,7 +26203,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="28" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B51" s="29"/>
       <c r="C51" s="29"/>
@@ -26204,7 +26229,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="30" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B52" s="33">
         <v>7.19</v>
@@ -26268,7 +26293,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="30" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B53" s="33">
         <v>11.46</v>
@@ -26324,7 +26349,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="28" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B54" s="29"/>
       <c r="C54" s="29"/>
@@ -26350,7 +26375,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="30" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B55" s="33">
         <v>7.78</v>
@@ -26414,7 +26439,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="30" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B56" s="33">
         <v>1.26</v>
@@ -26470,7 +26495,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="28" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B57" s="29"/>
       <c r="C57" s="29"/>
@@ -26496,7 +26521,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="30" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B58" s="33">
         <v>0.01</v>
@@ -26560,7 +26585,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="30" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B59" s="33">
         <v>0.68</v>
@@ -26616,7 +26641,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="28" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B60" s="29"/>
       <c r="C60" s="29"/>
@@ -26642,7 +26667,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="30" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B61" s="33">
         <v>1.21</v>
@@ -26706,7 +26731,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="30" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B62" s="33">
         <v>1.28</v>
@@ -26762,7 +26787,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="28" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B63" s="29"/>
       <c r="C63" s="29"/>
@@ -26788,7 +26813,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="30" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B64" s="33">
         <v>7.38</v>
@@ -26852,7 +26877,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="30" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B65" s="33">
         <v>7.59</v>
@@ -26908,7 +26933,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="28" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B66" s="29"/>
       <c r="C66" s="29"/>
@@ -26934,7 +26959,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="30" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B67" s="33">
         <v>17.14</v>
@@ -26998,7 +27023,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="30" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B68" s="33">
         <v>12.26</v>
@@ -27054,7 +27079,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="28" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B69" s="29"/>
       <c r="C69" s="29"/>
@@ -27080,7 +27105,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="30" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B70" s="32">
         <v>199.71</v>
@@ -27138,7 +27163,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="30" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B71" s="33">
         <v>28.91</v>

</xml_diff>